<commit_message>
[view&controller] update page register promotion
</commit_message>
<xml_diff>
--- a/NewShop/Excel/Order_Upload_By_Customer.xlsx
+++ b/NewShop/Excel/Order_Upload_By_Customer.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24931"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\work spaces\NewShop\NewShop\Excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\dotnet\NewShopGit\NewShop\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0713623-12FE-47FC-9399-6F99BF314FF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{424790C2-8BB6-4A79-BA7A-AD1C6345C036}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{7D3AAAC1-9BCF-4AB1-940E-4AC7DE0EFB5A}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{7D3AAAC1-9BCF-4AB1-940E-4AC7DE0EFB5A}"/>
   </bookViews>
   <sheets>
     <sheet name="Order" sheetId="1" r:id="rId1"/>
@@ -35,12 +35,18 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
   <si>
     <t>Qty</t>
   </si>
   <si>
-    <t>Item No.</t>
+    <t>Price</t>
+  </si>
+  <si>
+    <t>Company</t>
+  </si>
+  <si>
+    <t>Item No.2</t>
   </si>
 </sst>
 </file>
@@ -76,16 +82,25 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="5">
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -109,20 +124,22 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{F32448EE-C8BC-4149-83AF-8482C547C972}" name="Table2" displayName="Table2" ref="A1:B2" totalsRowShown="0" dataDxfId="2">
-  <autoFilter ref="A1:B2" xr:uid="{F32448EE-C8BC-4149-83AF-8482C547C972}"/>
-  <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{9021C813-B7D0-4991-B493-888F6353E8CF}" name="Item No." dataDxfId="1"/>
-    <tableColumn id="2" xr3:uid="{29D21503-10DD-4B74-9A0C-FF5B58E1E4B8}" name="Qty" dataDxfId="0"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{F32448EE-C8BC-4149-83AF-8482C547C972}" name="Table2" displayName="Table2" ref="A1:D2" insertRow="1" totalsRowShown="0" dataDxfId="4">
+  <autoFilter ref="A1:D2" xr:uid="{F32448EE-C8BC-4149-83AF-8482C547C972}"/>
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{9021C813-B7D0-4991-B493-888F6353E8CF}" name="Company" dataDxfId="3"/>
+    <tableColumn id="2" xr3:uid="{29D21503-10DD-4B74-9A0C-FF5B58E1E4B8}" name="Item No.2" dataDxfId="2"/>
+    <tableColumn id="3" xr3:uid="{AAF8CA41-4689-4AE8-AB89-763A620A1BF9}" name="Qty" dataDxfId="1"/>
+    <tableColumn id="4" xr3:uid="{CB40A1F6-1634-45B0-9F9E-3D79F964B79D}" name="Price" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -160,7 +177,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -266,7 +283,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -408,7 +425,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -416,22 +433,30 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE008E45-25F6-4E2B-9326-89F9C3155753}">
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.85546875" style="1" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" t="s">
         <v>1</v>
       </c>
-      <c r="B1" t="s">
-        <v>0</v>
-      </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
[view&controller] add function download excel result upload order
</commit_message>
<xml_diff>
--- a/NewShop/Excel/Order_Upload_By_Customer.xlsx
+++ b/NewShop/Excel/Order_Upload_By_Customer.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\dotnet\NewShopGit\NewShop\Excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\warakorn.pra\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{424790C2-8BB6-4A79-BA7A-AD1C6345C036}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{2CE992A7-FCC0-4F5D-AFFF-2F86BF5D69E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{7D3AAAC1-9BCF-4AB1-940E-4AC7DE0EFB5A}"/>
+    <workbookView xWindow="240" yWindow="480" windowWidth="28770" windowHeight="15570" xr2:uid="{C1047303-5F5A-490A-9785-8EB9F09762A0}"/>
   </bookViews>
   <sheets>
     <sheet name="Order" sheetId="1" r:id="rId1"/>
@@ -28,6 +28,7 @@
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
         <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -35,7 +36,10 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+  <si>
+    <t>Item No.</t>
+  </si>
   <si>
     <t>Qty</t>
   </si>
@@ -46,14 +50,14 @@
     <t>Company</t>
   </si>
   <si>
-    <t>Item No.2</t>
+    <t>Customer Part No.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -61,16 +65,30 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor theme="4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -78,34 +96,139 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </top>
+      <bottom style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="5">
     <dxf>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <font>
+        <sz val="18"/>
+        <color rgb="FF292B2C"/>
+        <name val="AngsanaUPC"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="right" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
     </dxf>
     <dxf>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <font>
+        <sz val="18"/>
+        <color rgb="FF292B2C"/>
+        <name val="AngsanaUPC"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
     </dxf>
     <dxf>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <numFmt numFmtId="30" formatCode="@"/>
     </dxf>
     <dxf>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <font>
+        <sz val="18"/>
+        <color rgb="FF292B2C"/>
+        <name val="AngsanaUPC"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
     </dxf>
     <dxf>
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -124,13 +247,14 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{F32448EE-C8BC-4149-83AF-8482C547C972}" name="Table2" displayName="Table2" ref="A1:D2" insertRow="1" totalsRowShown="0" dataDxfId="4">
-  <autoFilter ref="A1:D2" xr:uid="{F32448EE-C8BC-4149-83AF-8482C547C972}"/>
-  <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{9021C813-B7D0-4991-B493-888F6353E8CF}" name="Company" dataDxfId="3"/>
-    <tableColumn id="2" xr3:uid="{29D21503-10DD-4B74-9A0C-FF5B58E1E4B8}" name="Item No.2" dataDxfId="2"/>
-    <tableColumn id="3" xr3:uid="{AAF8CA41-4689-4AE8-AB89-763A620A1BF9}" name="Qty" dataDxfId="1"/>
-    <tableColumn id="4" xr3:uid="{CB40A1F6-1634-45B0-9F9E-3D79F964B79D}" name="Price" dataDxfId="0"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{C5EB0F5D-F096-4AB2-9C42-78E52111028C}" name="Table2" displayName="Table2" ref="A1:E2" insertRow="1" totalsRowShown="0">
+  <autoFilter ref="A1:E2" xr:uid="{F32448EE-C8BC-4149-83AF-8482C547C972}"/>
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{6C981F3E-F6B1-46D6-9F67-B1097E20EC2D}" name="Company" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{645FD8EF-DE42-4022-AF38-89DA92672B19}" name="Item No." dataDxfId="3"/>
+    <tableColumn id="5" xr3:uid="{10D0A77A-C748-4AF5-BA9C-182DBAF62EC8}" name="Customer Part No." dataDxfId="2"/>
+    <tableColumn id="3" xr3:uid="{8ED17FCC-A105-4816-BDE8-E58A4E46C29A}" name="Qty" dataDxfId="1"/>
+    <tableColumn id="4" xr3:uid="{0C1ED563-AD82-41A0-BC1F-8E2F9DBA2C1E}" name="Price" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -432,31 +556,35 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE008E45-25F6-4E2B-9326-89F9C3155753}">
-  <dimension ref="A1:D2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BB1AF864-61EA-40F4-9078-188F28439E25}">
+  <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.7109375" customWidth="1"/>
+    <col min="3" max="3" width="15.140625" style="4" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>2</v>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>3</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>3</v>
+        <v>0</v>
       </c>
-      <c r="C1" t="s">
-        <v>0</v>
+      <c r="C1" s="3" t="s">
+        <v>4</v>
       </c>
       <c r="D1" t="s">
         <v>1</v>
       </c>
+      <c r="E1" t="s">
+        <v>2</v>
+      </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
+      <c r="C2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
[controller&model] add module RBAC
</commit_message>
<xml_diff>
--- a/NewShop/Excel/Order_Upload_By_Customer.xlsx
+++ b/NewShop/Excel/Order_Upload_By_Customer.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\warakorn.pra\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\dotnet\NewShopGit\NewShop\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2CE992A7-FCC0-4F5D-AFFF-2F86BF5D69E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E03081A-62CB-4FF0-9BAC-837115BFB220}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="480" windowWidth="28770" windowHeight="15570" xr2:uid="{C1047303-5F5A-490A-9785-8EB9F09762A0}"/>
+    <workbookView xWindow="28800" yWindow="1740" windowWidth="21600" windowHeight="13335" xr2:uid="{C1047303-5F5A-490A-9785-8EB9F09762A0}"/>
   </bookViews>
   <sheets>
     <sheet name="Order" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>Item No.</t>
   </si>
@@ -51,6 +51,9 @@
   </si>
   <si>
     <t>Customer Part No.</t>
+  </si>
+  <si>
+    <t>LineNote</t>
   </si>
 </sst>
 </file>
@@ -88,7 +91,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -109,11 +112,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -125,6 +139,7 @@
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -247,14 +262,15 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{C5EB0F5D-F096-4AB2-9C42-78E52111028C}" name="Table2" displayName="Table2" ref="A1:E2" insertRow="1" totalsRowShown="0">
-  <autoFilter ref="A1:E2" xr:uid="{F32448EE-C8BC-4149-83AF-8482C547C972}"/>
-  <tableColumns count="5">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{C5EB0F5D-F096-4AB2-9C42-78E52111028C}" name="Table2" displayName="Table2" ref="A1:F2" insertRow="1" totalsRowShown="0">
+  <autoFilter ref="A1:F2" xr:uid="{F32448EE-C8BC-4149-83AF-8482C547C972}"/>
+  <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{6C981F3E-F6B1-46D6-9F67-B1097E20EC2D}" name="Company" dataDxfId="4"/>
     <tableColumn id="2" xr3:uid="{645FD8EF-DE42-4022-AF38-89DA92672B19}" name="Item No." dataDxfId="3"/>
     <tableColumn id="5" xr3:uid="{10D0A77A-C748-4AF5-BA9C-182DBAF62EC8}" name="Customer Part No." dataDxfId="2"/>
     <tableColumn id="3" xr3:uid="{8ED17FCC-A105-4816-BDE8-E58A4E46C29A}" name="Qty" dataDxfId="1"/>
     <tableColumn id="4" xr3:uid="{0C1ED563-AD82-41A0-BC1F-8E2F9DBA2C1E}" name="Price" dataDxfId="0"/>
+    <tableColumn id="6" xr3:uid="{191607CA-9849-42D4-9016-EF4E08E0E65F}" name="LineNote"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -557,15 +573,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BB1AF864-61EA-40F4-9078-188F28439E25}">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13.7109375" customWidth="1"/>
     <col min="3" max="3" width="15.140625" style="4" customWidth="1"/>
+    <col min="6" max="6" width="12.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>3</v>
       </c>
@@ -581,8 +598,11 @@
       <c r="E1" t="s">
         <v>2</v>
       </c>
+      <c r="F1" s="5" t="s">
+        <v>5</v>
+      </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2"/>
       <c r="C2"/>
     </row>

</xml_diff>